<commit_message>
Mejoras en grabacion de aplicacion de comprobantes de proveedores
</commit_message>
<xml_diff>
--- a/resources/templates/caja/flash/plantilla-flash-agg.xlsx
+++ b/resources/templates/caja/flash/plantilla-flash-agg.xlsx
@@ -6660,56 +6660,56 @@
   <dimension ref="A1:BP59"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" style="39" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" style="39" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" style="39" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" style="39" customWidth="1"/>
     <col min="4" max="4" width="5" style="39" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.88671875" style="39" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10" style="39" customWidth="1"/>
-    <col min="8" max="8" width="7.140625" style="39" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" style="39" customWidth="1"/>
-    <col min="10" max="10" width="6.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.109375" style="39" customWidth="1"/>
+    <col min="9" max="9" width="6.33203125" style="39" customWidth="1"/>
+    <col min="10" max="10" width="6.5546875" style="39" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8" style="39" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.28515625" style="39" customWidth="1"/>
-    <col min="13" max="13" width="11.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.33203125" style="39" customWidth="1"/>
+    <col min="13" max="13" width="11.33203125" style="39" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.109375" style="39" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.5703125" style="39" customWidth="1"/>
-    <col min="18" max="18" width="7.42578125" style="39" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.44140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.5546875" style="39" customWidth="1"/>
+    <col min="18" max="18" width="7.44140625" style="39" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="8" style="39" customWidth="1"/>
-    <col min="20" max="20" width="10.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.42578125" style="39" customWidth="1"/>
-    <col min="22" max="22" width="6.5703125" style="39" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="11.140625" style="39" hidden="1" customWidth="1"/>
-    <col min="24" max="25" width="10.140625" style="39" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="8.85546875" style="39" hidden="1" customWidth="1"/>
-    <col min="27" max="29" width="6.5703125" style="39" hidden="1" customWidth="1"/>
-    <col min="30" max="32" width="10.7109375" style="39" customWidth="1"/>
-    <col min="33" max="33" width="9.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.140625" style="39" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="6.28515625" style="39" customWidth="1"/>
-    <col min="37" max="37" width="10.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="38" max="39" width="9.42578125" style="39" customWidth="1"/>
-    <col min="40" max="41" width="9.140625" style="39" customWidth="1"/>
-    <col min="42" max="42" width="7.28515625" style="39" customWidth="1"/>
-    <col min="43" max="43" width="11.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="10.85546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.44140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.44140625" style="39" customWidth="1"/>
+    <col min="22" max="22" width="6.5546875" style="39" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="11.109375" style="39" hidden="1" customWidth="1"/>
+    <col min="24" max="25" width="10.109375" style="39" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="8.88671875" style="39" hidden="1" customWidth="1"/>
+    <col min="27" max="29" width="6.5546875" style="39" hidden="1" customWidth="1"/>
+    <col min="30" max="32" width="10.6640625" style="39" customWidth="1"/>
+    <col min="33" max="33" width="9.109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.109375" style="39" customWidth="1"/>
+    <col min="35" max="35" width="9.109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="6.33203125" style="39" customWidth="1"/>
+    <col min="37" max="37" width="10.88671875" style="39" bestFit="1" customWidth="1"/>
+    <col min="38" max="39" width="9.44140625" style="39" customWidth="1"/>
+    <col min="40" max="41" width="9.109375" style="39" customWidth="1"/>
+    <col min="42" max="42" width="7.33203125" style="39" customWidth="1"/>
+    <col min="43" max="43" width="11.109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.88671875" style="39" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10.5546875" style="39" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="12.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="7.28515625" style="39" customWidth="1"/>
-    <col min="50" max="50" width="4.5703125" style="39" customWidth="1"/>
-    <col min="51" max="56" width="8.7109375" style="39" customWidth="1"/>
-    <col min="57" max="57" width="10.5703125" style="39" customWidth="1"/>
-    <col min="58" max="61" width="10.7109375" style="39" customWidth="1"/>
-    <col min="62" max="62" width="10.5703125" style="39" customWidth="1"/>
-    <col min="63" max="66" width="10.7109375" style="39" customWidth="1"/>
-    <col min="67" max="75" width="11.42578125" style="39" customWidth="1"/>
-    <col min="76" max="16384" width="11.42578125" style="39"/>
+    <col min="48" max="48" width="12.5546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="7.33203125" style="39" customWidth="1"/>
+    <col min="50" max="50" width="4.5546875" style="39" customWidth="1"/>
+    <col min="51" max="56" width="8.6640625" style="39" customWidth="1"/>
+    <col min="57" max="57" width="10.5546875" style="39" customWidth="1"/>
+    <col min="58" max="61" width="10.6640625" style="39" customWidth="1"/>
+    <col min="62" max="62" width="10.5546875" style="39" customWidth="1"/>
+    <col min="63" max="66" width="10.6640625" style="39" customWidth="1"/>
+    <col min="67" max="75" width="11.44140625" style="39" customWidth="1"/>
+    <col min="76" max="16384" width="11.44140625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:68" x14ac:dyDescent="0.2">
@@ -18104,63 +18104,63 @@
   <dimension ref="C8:BK37"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="21" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="7" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="6" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="6" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="11" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="20.5546875" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="7" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="6" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="44" max="45" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="7" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="52" max="53" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="6" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="52" max="54" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="58" max="58" width="9" bestFit="1" customWidth="1"/>
-    <col min="59" max="60" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="10" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="63" max="63" width="9" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="8" spans="5:63" x14ac:dyDescent="0.2">
@@ -18536,60 +18536,60 @@
   <dimension ref="A1:BX60"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" style="39" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="39" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" style="39" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="10.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.140625" style="39" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" style="39" customWidth="1"/>
-    <col min="10" max="10" width="6.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" style="39" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" style="39" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" style="39" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="10.88671875" style="39" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.109375" style="39" customWidth="1"/>
+    <col min="9" max="9" width="6.33203125" style="39" customWidth="1"/>
+    <col min="10" max="10" width="6.5546875" style="39" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8" style="39" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.28515625" style="39" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.5703125" style="39" customWidth="1"/>
-    <col min="18" max="18" width="7.42578125" style="39" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.33203125" style="39" customWidth="1"/>
+    <col min="13" max="13" width="11.6640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.88671875" style="39" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.5546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.44140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.5546875" style="39" customWidth="1"/>
+    <col min="18" max="18" width="7.44140625" style="39" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="8" style="39" customWidth="1"/>
-    <col min="20" max="20" width="10.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.42578125" style="39" customWidth="1"/>
-    <col min="22" max="22" width="6.5703125" style="39" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="11.140625" style="39" hidden="1" customWidth="1"/>
-    <col min="24" max="25" width="10.140625" style="39" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="8.85546875" style="39" hidden="1" customWidth="1"/>
-    <col min="27" max="29" width="6.5703125" style="39" hidden="1" customWidth="1"/>
-    <col min="30" max="32" width="10.7109375" style="39" customWidth="1"/>
-    <col min="33" max="33" width="9.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.140625" style="39" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="6.28515625" style="39" customWidth="1"/>
-    <col min="37" max="37" width="10.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="9.7109375" style="39" customWidth="1"/>
-    <col min="39" max="42" width="9.42578125" style="39" customWidth="1"/>
-    <col min="43" max="43" width="11.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="10.85546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.44140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.44140625" style="39" customWidth="1"/>
+    <col min="22" max="22" width="6.5546875" style="39" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="11.109375" style="39" hidden="1" customWidth="1"/>
+    <col min="24" max="25" width="10.109375" style="39" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="8.88671875" style="39" hidden="1" customWidth="1"/>
+    <col min="27" max="29" width="6.5546875" style="39" hidden="1" customWidth="1"/>
+    <col min="30" max="32" width="10.6640625" style="39" customWidth="1"/>
+    <col min="33" max="33" width="9.109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.109375" style="39" customWidth="1"/>
+    <col min="35" max="35" width="9.109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="6.33203125" style="39" customWidth="1"/>
+    <col min="37" max="37" width="10.88671875" style="39" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="9.6640625" style="39" customWidth="1"/>
+    <col min="39" max="42" width="9.44140625" style="39" customWidth="1"/>
+    <col min="43" max="43" width="11.109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.88671875" style="39" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10.5546875" style="39" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="12.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="7.28515625" style="39" customWidth="1"/>
-    <col min="50" max="50" width="4.5703125" style="39" customWidth="1"/>
-    <col min="51" max="56" width="8.7109375" style="39" customWidth="1"/>
+    <col min="48" max="48" width="12.5546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="7.33203125" style="39" customWidth="1"/>
+    <col min="50" max="50" width="4.5546875" style="39" customWidth="1"/>
+    <col min="51" max="56" width="8.6640625" style="39" customWidth="1"/>
     <col min="57" max="58" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="7.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="60" max="61" width="9.42578125" style="39" customWidth="1"/>
-    <col min="62" max="62" width="11.5703125" style="39" customWidth="1"/>
+    <col min="59" max="59" width="7.88671875" style="39" bestFit="1" customWidth="1"/>
+    <col min="60" max="61" width="9.44140625" style="39" customWidth="1"/>
+    <col min="62" max="62" width="11.5546875" style="39" customWidth="1"/>
     <col min="63" max="63" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="64" max="66" width="9.42578125" style="39" customWidth="1"/>
-    <col min="67" max="67" width="10.140625" style="39" customWidth="1"/>
-    <col min="68" max="76" width="11.42578125" style="39" hidden="1" customWidth="1"/>
-    <col min="77" max="77" width="11.42578125" style="39" customWidth="1"/>
-    <col min="78" max="78" width="11.28515625" style="39" customWidth="1"/>
-    <col min="79" max="94" width="11.42578125" style="39" customWidth="1"/>
-    <col min="95" max="16384" width="11.42578125" style="39"/>
+    <col min="64" max="66" width="9.44140625" style="39" customWidth="1"/>
+    <col min="67" max="67" width="10.109375" style="39" customWidth="1"/>
+    <col min="68" max="76" width="11.44140625" style="39" hidden="1" customWidth="1"/>
+    <col min="77" max="77" width="11.44140625" style="39" customWidth="1"/>
+    <col min="78" max="78" width="11.33203125" style="39" customWidth="1"/>
+    <col min="79" max="94" width="11.44140625" style="39" customWidth="1"/>
+    <col min="95" max="16384" width="11.44140625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:68" x14ac:dyDescent="0.2">
@@ -29948,58 +29948,58 @@
   <dimension ref="A1:BX60"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" style="39" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="39" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" style="39" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.140625" style="39" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" style="39" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" style="39" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" style="39" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" style="39" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.109375" style="39" customWidth="1"/>
     <col min="7" max="7" width="10" style="39" customWidth="1"/>
-    <col min="8" max="8" width="7.140625" style="39" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" style="39" customWidth="1"/>
-    <col min="10" max="10" width="6.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.109375" style="39" customWidth="1"/>
+    <col min="9" max="9" width="6.33203125" style="39" customWidth="1"/>
+    <col min="10" max="10" width="6.5546875" style="39" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8" style="39" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.28515625" style="39" customWidth="1"/>
-    <col min="13" max="13" width="11.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.33203125" style="39" customWidth="1"/>
+    <col min="13" max="13" width="11.33203125" style="39" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.109375" style="39" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.5703125" style="39" customWidth="1"/>
-    <col min="18" max="18" width="7.42578125" style="39" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.44140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.5546875" style="39" customWidth="1"/>
+    <col min="18" max="18" width="7.44140625" style="39" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="8" style="39" customWidth="1"/>
-    <col min="20" max="20" width="10.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.42578125" style="39" customWidth="1"/>
-    <col min="22" max="22" width="6.5703125" style="39" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="11.140625" style="39" hidden="1" customWidth="1"/>
-    <col min="24" max="25" width="10.140625" style="39" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="8.85546875" style="39" hidden="1" customWidth="1"/>
-    <col min="27" max="29" width="6.5703125" style="39" hidden="1" customWidth="1"/>
-    <col min="30" max="32" width="10.7109375" style="39" customWidth="1"/>
-    <col min="33" max="35" width="9.140625" style="39" customWidth="1"/>
-    <col min="36" max="36" width="6.28515625" style="39" customWidth="1"/>
-    <col min="37" max="37" width="10.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="38" max="42" width="9.42578125" style="39" customWidth="1"/>
-    <col min="43" max="43" width="11.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="10.85546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.44140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.44140625" style="39" customWidth="1"/>
+    <col min="22" max="22" width="6.5546875" style="39" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="11.109375" style="39" hidden="1" customWidth="1"/>
+    <col min="24" max="25" width="10.109375" style="39" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="8.88671875" style="39" hidden="1" customWidth="1"/>
+    <col min="27" max="29" width="6.5546875" style="39" hidden="1" customWidth="1"/>
+    <col min="30" max="32" width="10.6640625" style="39" customWidth="1"/>
+    <col min="33" max="35" width="9.109375" style="39" customWidth="1"/>
+    <col min="36" max="36" width="6.33203125" style="39" customWidth="1"/>
+    <col min="37" max="37" width="10.44140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="38" max="42" width="9.44140625" style="39" customWidth="1"/>
+    <col min="43" max="43" width="11.109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.88671875" style="39" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10.5546875" style="39" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="12.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="7.28515625" style="39" customWidth="1"/>
-    <col min="50" max="50" width="4.5703125" style="39" customWidth="1"/>
-    <col min="51" max="56" width="8.7109375" style="39" customWidth="1"/>
-    <col min="57" max="57" width="11.5703125" style="39" customWidth="1"/>
+    <col min="48" max="48" width="12.5546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="7.33203125" style="39" customWidth="1"/>
+    <col min="50" max="50" width="4.5546875" style="39" customWidth="1"/>
+    <col min="51" max="56" width="8.6640625" style="39" customWidth="1"/>
+    <col min="57" max="57" width="11.5546875" style="39" customWidth="1"/>
     <col min="58" max="58" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="59" max="61" width="9.42578125" style="39" customWidth="1"/>
-    <col min="62" max="62" width="11.5703125" style="39" customWidth="1"/>
+    <col min="59" max="61" width="9.44140625" style="39" customWidth="1"/>
+    <col min="62" max="62" width="11.5546875" style="39" customWidth="1"/>
     <col min="63" max="63" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="64" max="66" width="9.42578125" style="39" customWidth="1"/>
-    <col min="67" max="67" width="11.42578125" style="39"/>
-    <col min="68" max="76" width="11.42578125" style="39" hidden="1" customWidth="1"/>
-    <col min="77" max="77" width="11.42578125" style="39" customWidth="1"/>
-    <col min="78" max="78" width="11.28515625" style="39" customWidth="1"/>
-    <col min="79" max="79" width="11.42578125" style="39" customWidth="1"/>
-    <col min="80" max="16384" width="11.42578125" style="39"/>
+    <col min="64" max="66" width="9.44140625" style="39" customWidth="1"/>
+    <col min="67" max="67" width="11.44140625" style="39"/>
+    <col min="68" max="76" width="11.44140625" style="39" hidden="1" customWidth="1"/>
+    <col min="77" max="77" width="11.44140625" style="39" customWidth="1"/>
+    <col min="78" max="78" width="11.33203125" style="39" customWidth="1"/>
+    <col min="79" max="79" width="11.44140625" style="39" customWidth="1"/>
+    <col min="80" max="16384" width="11.44140625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:68" x14ac:dyDescent="0.2">
@@ -41173,64 +41173,64 @@
   <dimension ref="A1:BX60"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" style="39" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="39" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" style="39" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.140625" style="39" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" style="39" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" style="39" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" style="39" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" style="39" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.109375" style="39" customWidth="1"/>
     <col min="7" max="7" width="10" style="39" customWidth="1"/>
-    <col min="8" max="8" width="7.140625" style="39" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" style="39" customWidth="1"/>
-    <col min="10" max="10" width="6.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.109375" style="39" customWidth="1"/>
+    <col min="9" max="9" width="6.33203125" style="39" customWidth="1"/>
+    <col min="10" max="10" width="6.5546875" style="39" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8" style="39" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.28515625" style="39" customWidth="1"/>
-    <col min="13" max="13" width="11.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.33203125" style="39" customWidth="1"/>
+    <col min="13" max="13" width="11.33203125" style="39" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.109375" style="39" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.5703125" style="39" customWidth="1"/>
-    <col min="18" max="18" width="7.42578125" style="39" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.44140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.5546875" style="39" customWidth="1"/>
+    <col min="18" max="18" width="7.44140625" style="39" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="8" style="39" customWidth="1"/>
-    <col min="20" max="20" width="10.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.42578125" style="39" customWidth="1"/>
-    <col min="22" max="22" width="6.5703125" style="39" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="11.140625" style="39" hidden="1" customWidth="1"/>
-    <col min="24" max="25" width="10.140625" style="39" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="8.85546875" style="39" hidden="1" customWidth="1"/>
-    <col min="27" max="29" width="6.5703125" style="39" hidden="1" customWidth="1"/>
-    <col min="30" max="32" width="10.7109375" style="39" customWidth="1"/>
-    <col min="33" max="33" width="9.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.140625" style="39" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="6.28515625" style="39" customWidth="1"/>
-    <col min="37" max="37" width="10.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="38" max="39" width="9.42578125" style="39" customWidth="1"/>
-    <col min="40" max="40" width="14.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="41" max="42" width="9.42578125" style="39" customWidth="1"/>
-    <col min="43" max="43" width="11.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="10.85546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.44140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.44140625" style="39" customWidth="1"/>
+    <col min="22" max="22" width="6.5546875" style="39" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="11.109375" style="39" hidden="1" customWidth="1"/>
+    <col min="24" max="25" width="10.109375" style="39" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="8.88671875" style="39" hidden="1" customWidth="1"/>
+    <col min="27" max="29" width="6.5546875" style="39" hidden="1" customWidth="1"/>
+    <col min="30" max="32" width="10.6640625" style="39" customWidth="1"/>
+    <col min="33" max="33" width="9.109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.109375" style="39" customWidth="1"/>
+    <col min="35" max="35" width="9.109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="6.33203125" style="39" customWidth="1"/>
+    <col min="37" max="37" width="10.44140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="38" max="39" width="9.44140625" style="39" customWidth="1"/>
+    <col min="40" max="40" width="14.44140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="41" max="42" width="9.44140625" style="39" customWidth="1"/>
+    <col min="43" max="43" width="11.109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.88671875" style="39" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10.5546875" style="39" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="12.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="7.28515625" style="39" customWidth="1"/>
-    <col min="50" max="50" width="4.5703125" style="39" customWidth="1"/>
-    <col min="51" max="52" width="8.7109375" style="39" customWidth="1"/>
+    <col min="48" max="48" width="12.5546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="7.33203125" style="39" customWidth="1"/>
+    <col min="50" max="50" width="4.5546875" style="39" customWidth="1"/>
+    <col min="51" max="52" width="8.6640625" style="39" customWidth="1"/>
     <col min="53" max="53" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="54" max="56" width="8.7109375" style="39" customWidth="1"/>
-    <col min="57" max="57" width="11.5703125" style="39" customWidth="1"/>
+    <col min="54" max="56" width="8.6640625" style="39" customWidth="1"/>
+    <col min="57" max="57" width="11.5546875" style="39" customWidth="1"/>
     <col min="58" max="58" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="59" max="61" width="9.42578125" style="39" customWidth="1"/>
-    <col min="62" max="62" width="11.5703125" style="39" customWidth="1"/>
+    <col min="59" max="61" width="9.44140625" style="39" customWidth="1"/>
+    <col min="62" max="62" width="11.5546875" style="39" customWidth="1"/>
     <col min="63" max="63" width="10" style="39" bestFit="1" customWidth="1"/>
-    <col min="64" max="66" width="9.42578125" style="39" customWidth="1"/>
-    <col min="67" max="67" width="11.42578125" style="39"/>
-    <col min="68" max="76" width="11.42578125" style="39" hidden="1" customWidth="1"/>
-    <col min="77" max="77" width="11.42578125" style="39" customWidth="1"/>
-    <col min="78" max="78" width="11.28515625" style="39" customWidth="1"/>
-    <col min="79" max="79" width="11.42578125" style="39" customWidth="1"/>
-    <col min="80" max="16384" width="11.42578125" style="39"/>
+    <col min="64" max="66" width="9.44140625" style="39" customWidth="1"/>
+    <col min="67" max="67" width="11.44140625" style="39"/>
+    <col min="68" max="76" width="11.44140625" style="39" hidden="1" customWidth="1"/>
+    <col min="77" max="77" width="11.44140625" style="39" customWidth="1"/>
+    <col min="78" max="78" width="11.33203125" style="39" customWidth="1"/>
+    <col min="79" max="79" width="11.44140625" style="39" customWidth="1"/>
+    <col min="80" max="16384" width="11.44140625" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:68" x14ac:dyDescent="0.2">
@@ -52374,19 +52374,18 @@
   <dimension ref="A2:M23"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="145" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" style="145" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="145" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7109375" style="145" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" style="145" customWidth="1"/>
-    <col min="6" max="6" width="3.42578125" style="145" customWidth="1"/>
-    <col min="7" max="8" width="13.7109375" style="145" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="4.85546875" style="145" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" style="145" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="145" customWidth="1"/>
-    <col min="12" max="12" width="16.42578125" style="145" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" style="145" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" style="145" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" style="145" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" style="145" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" style="145" customWidth="1"/>
+    <col min="6" max="6" width="3.44140625" style="145" customWidth="1"/>
+    <col min="7" max="8" width="13.6640625" style="145" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="4.88671875" style="145" hidden="1" customWidth="1"/>
+    <col min="10" max="11" width="13.6640625" style="145" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="16.44140625" style="145" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="7" style="154" customWidth="1"/>
-    <col min="14" max="16384" width="11.42578125" style="145"/>
+    <col min="14" max="16384" width="11.44140625" style="145"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
@@ -52634,18 +52633,18 @@
   <dimension ref="B2:T215"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="11.42578125" style="39"/>
+    <col min="1" max="2" width="11.44140625" style="39"/>
     <col min="3" max="3" width="13" style="39" customWidth="1"/>
-    <col min="4" max="5" width="12.7109375" style="39" customWidth="1"/>
-    <col min="6" max="10" width="11.42578125" style="39"/>
+    <col min="4" max="5" width="12.6640625" style="39" customWidth="1"/>
+    <col min="6" max="10" width="11.44140625" style="39"/>
     <col min="11" max="11" width="13" style="39" customWidth="1"/>
-    <col min="12" max="12" width="12.140625" style="39" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" style="39" customWidth="1"/>
-    <col min="14" max="14" width="12.85546875" style="39" customWidth="1"/>
-    <col min="15" max="18" width="11.42578125" style="39"/>
-    <col min="19" max="19" width="12.28515625" style="39" customWidth="1"/>
-    <col min="20" max="20" width="12.85546875" style="39" customWidth="1"/>
-    <col min="21" max="16384" width="11.42578125" style="39"/>
+    <col min="12" max="12" width="12.109375" style="39" customWidth="1"/>
+    <col min="13" max="13" width="12.6640625" style="39" customWidth="1"/>
+    <col min="14" max="14" width="12.88671875" style="39" customWidth="1"/>
+    <col min="15" max="18" width="11.44140625" style="39"/>
+    <col min="19" max="19" width="12.33203125" style="39" customWidth="1"/>
+    <col min="20" max="20" width="12.88671875" style="39" customWidth="1"/>
+    <col min="21" max="16384" width="11.44140625" style="39"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.2">
@@ -59918,61 +59917,62 @@
   <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="21" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="7" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="6" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="6" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="7" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="11" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="20.5546875" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="7" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="6" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="44" max="45" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="48" max="48" width="7" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="52" max="53" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="52" max="53" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="10" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="58" max="58" width="9" bestFit="1" customWidth="1"/>
-    <col min="59" max="60" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="60" width="10" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="63" max="63" width="9" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="9" spans="5:63" x14ac:dyDescent="0.2">
@@ -60347,63 +60347,63 @@
   <dimension ref="C8:BK37"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="21" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="7" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="6" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="6" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="6" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="7" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="7" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="6" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="44" max="45" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="7" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="52" max="53" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="45" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="6" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="52" max="53" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="58" max="58" width="9" bestFit="1" customWidth="1"/>
-    <col min="59" max="60" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="60" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="63" max="63" width="9" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="8" spans="5:63" x14ac:dyDescent="0.2">
@@ -60779,61 +60779,65 @@
   <dimension ref="C8:BK37"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="21" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="7" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="6" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="6" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="6" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="11" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="7" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="6" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="44" max="45" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="7" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="52" max="53" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="45" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="6" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="52" max="53" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="9.109375" bestFit="1" customWidth="1"/>
     <col min="58" max="58" width="9" bestFit="1" customWidth="1"/>
-    <col min="59" max="60" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="60" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="63" max="63" width="9" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="8" spans="5:63" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Modificaciones en emisor del mayor, mejoras en cumple requi de sala sin NPU, iva digital
</commit_message>
<xml_diff>
--- a/resources/templates/caja/flash/plantilla-flash-agg.xlsx
+++ b/resources/templates/caja/flash/plantilla-flash-agg.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="137">
   <si>
     <t>Consolidated Income</t>
   </si>
@@ -447,6 +447,12 @@
   </si>
   <si>
     <t>Reporte Flash Agosto 25</t>
+  </si>
+  <si>
+    <t>Slots</t>
+  </si>
+  <si>
+    <t>Ruletas</t>
   </si>
 </sst>
 </file>
@@ -52371,255 +52377,335 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A2:M23"/>
+  <dimension ref="A2:O23"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.6640625" style="145" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5546875" style="145" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.109375" style="145" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.6640625" style="145" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" style="145" customWidth="1"/>
-    <col min="6" max="6" width="3.44140625" style="145" customWidth="1"/>
-    <col min="7" max="8" width="13.6640625" style="145" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="4.88671875" style="145" hidden="1" customWidth="1"/>
-    <col min="10" max="11" width="13.6640625" style="145" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="16.44140625" style="145" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="7" style="154" customWidth="1"/>
-    <col min="14" max="16384" width="11.44140625" style="145"/>
+    <col min="2" max="3" width="9.5546875" style="145" customWidth="1"/>
+    <col min="4" max="4" width="9.5546875" style="145" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" style="145" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" style="145" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" style="145" customWidth="1"/>
+    <col min="8" max="8" width="3.44140625" style="145" customWidth="1"/>
+    <col min="9" max="10" width="13.6640625" style="145" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="4.88671875" style="145" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" style="145" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="13.6640625" style="145" customWidth="1"/>
+    <col min="14" max="14" width="16.44140625" style="145" customWidth="1"/>
+    <col min="15" max="15" width="7" style="154" customWidth="1"/>
+    <col min="16" max="16384" width="11.44140625" style="145"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="160" t="s">
         <v>92</v>
       </c>
       <c r="B2" s="161" t="s">
+        <v>135</v>
+      </c>
+      <c r="C2" s="161" t="s">
+        <v>136</v>
+      </c>
+      <c r="D2" s="161" t="s">
         <v>87</v>
       </c>
-      <c r="C2" s="161"/>
-      <c r="D2" s="161"/>
+      <c r="E2" s="161"/>
+      <c r="F2" s="161"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="155" t="s">
         <v>88</v>
       </c>
       <c r="B3" s="156">
-        <f>HLOOKUP(H3,Resumen!BE5:BH39,+'Biyemas S.A.'!D1+2,0)</f>
+        <f>SUM(B4:B6)</f>
         <v>0</v>
       </c>
-      <c r="D3" s="39"/>
-      <c r="G3" s="331" t="s">
+      <c r="C3" s="156">
+        <f>SUM(C4:C6)</f>
+        <v>0</v>
+      </c>
+      <c r="D3" s="156">
+        <f>HLOOKUP(J3,Resumen!BE5:BH39,+'Biyemas S.A.'!D1+2,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F3" s="39"/>
+      <c r="I3" s="331" t="s">
         <v>39</v>
       </c>
-      <c r="H3" s="289" t="s">
+      <c r="J3" s="289" t="s">
         <v>42</v>
       </c>
-      <c r="I3" s="289" t="s">
+      <c r="K3" s="289" t="s">
         <v>43</v>
       </c>
-      <c r="J3" s="333" t="s">
+      <c r="L3" s="333" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="155" t="s">
         <v>89</v>
       </c>
       <c r="B4" s="156">
-        <f>HLOOKUP(H3,'Biyemas S.A.'!BE5:BH39,+'Biyemas S.A.'!D1+2,0)</f>
+        <f>INDEX('Biyemas S.A.'!G7:G37,'Biyemas S.A.'!D1)</f>
         <v>0</v>
       </c>
-      <c r="D4" s="39"/>
-      <c r="G4" s="332"/>
-      <c r="H4" s="290"/>
-      <c r="I4" s="290"/>
-      <c r="J4" s="334"/>
+      <c r="C4" s="156">
+        <f>INDEX('Biyemas S.A.'!O7:O37,'Biyemas S.A.'!D1)</f>
+        <v>0</v>
+      </c>
+      <c r="D4" s="156">
+        <f>HLOOKUP(J3,'Biyemas S.A.'!BE5:BH39,+'Biyemas S.A.'!D1+2,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="39"/>
+      <c r="I4" s="332"/>
+      <c r="J4" s="290"/>
+      <c r="K4" s="290"/>
+      <c r="L4" s="334"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="155" t="s">
         <v>90</v>
       </c>
       <c r="B5" s="156">
-        <f>HLOOKUP(H3,'Kandiko S.A'!BA5:BF39,+'Biyemas S.A.'!D1+2,0)</f>
+        <f>INDEX('Kandiko S.A'!G7:G37,'Kandiko S.A'!D1)</f>
         <v>0</v>
       </c>
-      <c r="D5" s="39"/>
+      <c r="C5" s="156">
+        <f>INDEX('Kandiko S.A'!O7:O37,'Kandiko S.A'!D1)</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="156">
+        <f>HLOOKUP(J3,'Kandiko S.A'!BA5:BF39,+'Biyemas S.A.'!D1+2,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="39"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="155" t="s">
         <v>91</v>
       </c>
       <c r="B6" s="156">
-        <f>HLOOKUP(H3,'Rebisco S.A.'!BA5:BF39,+'Biyemas S.A.'!D1+2,0)</f>
+        <f>INDEX('Rebisco S.A.'!G7:G37,'Rebisco S.A.'!D1)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="39"/>
+      <c r="C6" s="156">
+        <f>INDEX('Rebisco S.A.'!O7:O37,'Rebisco S.A.'!D1)</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="156">
+        <f>HLOOKUP(J3,'Rebisco S.A.'!BA5:BF39,+'Biyemas S.A.'!D1+2,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="39"/>
     </row>
-    <row r="7" spans="1:13" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="157"/>
       <c r="B7" s="158"/>
       <c r="C7" s="158"/>
-      <c r="D7" s="39"/>
+      <c r="D7" s="158"/>
+      <c r="E7" s="158"/>
+      <c r="F7" s="39"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="160" t="s">
         <v>93</v>
       </c>
       <c r="B8" s="164" t="s">
+        <v>135</v>
+      </c>
+      <c r="C8" s="164" t="s">
+        <v>136</v>
+      </c>
+      <c r="D8" s="164" t="s">
         <v>87</v>
       </c>
-      <c r="C8" s="161" t="s">
+      <c r="E8" s="161" t="s">
         <v>118</v>
       </c>
-      <c r="D8" s="161" t="s">
+      <c r="F8" s="161" t="s">
         <v>119</v>
       </c>
-      <c r="L8" s="157"/>
-      <c r="M8" s="162"/>
+      <c r="N8" s="157"/>
+      <c r="O8" s="162"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="155" t="s">
         <v>88</v>
       </c>
-      <c r="B9" s="156" t="e">
+      <c r="B9" s="156">
+        <f>SUM(B10:B12)</f>
+        <v>0</v>
+      </c>
+      <c r="C9" s="156">
+        <f>SUM(C10:C12)</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="156" t="e">
         <f>+Resumen!BF39</f>
         <v>#N/A</v>
       </c>
-      <c r="C9" s="156" t="e">
+      <c r="E9" s="156" t="e">
         <f>+Resumen!AD48</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D9" s="156" t="e">
+      <c r="F9" s="156" t="e">
         <f>+Resumen!AD57</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="L9" s="157"/>
-      <c r="M9" s="163"/>
+      <c r="N9" s="157"/>
+      <c r="O9" s="163"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="155" t="s">
         <v>89</v>
       </c>
-      <c r="B10" s="156" t="e">
+      <c r="B10" s="156">
+        <f>+'Biyemas S.A.'!G39</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="156">
+        <f>+'Biyemas S.A.'!O39</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="156" t="e">
         <f>+'Biyemas S.A.'!BF39</f>
         <v>#N/A</v>
       </c>
-      <c r="C10" s="156" t="e">
+      <c r="E10" s="156" t="e">
         <f>+'Biyemas S.A.'!AD48</f>
         <v>#N/A</v>
       </c>
-      <c r="D10" s="156" t="e">
+      <c r="F10" s="156" t="e">
         <f>+'Biyemas S.A.'!AD57</f>
         <v>#N/A</v>
       </c>
-      <c r="L10" s="157"/>
-      <c r="M10" s="163"/>
+      <c r="N10" s="157"/>
+      <c r="O10" s="163"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="155" t="s">
         <v>90</v>
       </c>
-      <c r="B11" s="156" t="e">
+      <c r="B11" s="156">
+        <f>+'Kandiko S.A'!G39</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="156">
+        <f>+'Kandiko S.A'!O39</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="156" t="e">
         <f>+'Kandiko S.A'!BF39</f>
         <v>#N/A</v>
       </c>
-      <c r="C11" s="156" t="e">
+      <c r="E11" s="156" t="e">
         <f>+'Kandiko S.A'!AD48</f>
         <v>#N/A</v>
       </c>
-      <c r="D11" s="156" t="e">
+      <c r="F11" s="156" t="e">
         <f>+'Kandiko S.A'!AD57</f>
         <v>#N/A</v>
       </c>
-      <c r="L11" s="157"/>
-      <c r="M11" s="163"/>
+      <c r="N11" s="157"/>
+      <c r="O11" s="163"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="155" t="s">
         <v>91</v>
       </c>
-      <c r="B12" s="156" t="e">
+      <c r="B12" s="156">
+        <f>+'Rebisco S.A.'!G39</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="156">
+        <f>+'Rebisco S.A.'!O39</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="156" t="e">
         <f>+'Rebisco S.A.'!BF39</f>
         <v>#N/A</v>
       </c>
-      <c r="C12" s="156" t="e">
+      <c r="E12" s="156" t="e">
         <f>+'Rebisco S.A.'!AD48</f>
         <v>#N/A</v>
       </c>
-      <c r="D12" s="156" t="e">
+      <c r="F12" s="156" t="e">
         <f>+'Rebisco S.A.'!AD57</f>
         <v>#N/A</v>
       </c>
-      <c r="L12" s="157"/>
-      <c r="M12" s="163"/>
+      <c r="N12" s="157"/>
+      <c r="O12" s="163"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="39"/>
-      <c r="B13" s="39"/>
-      <c r="C13" s="39"/>
-      <c r="J13" s="160"/>
-      <c r="K13" s="161"/>
-      <c r="L13" s="157"/>
-      <c r="M13" s="159"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="L13" s="160"/>
+      <c r="M13" s="161"/>
+      <c r="N13" s="157"/>
+      <c r="O13" s="159"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
-      <c r="C14" s="39"/>
-      <c r="J14" s="155"/>
-      <c r="K14" s="156"/>
-      <c r="L14" s="157"/>
-      <c r="M14" s="162"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="L14" s="155"/>
+      <c r="M14" s="156"/>
+      <c r="N14" s="157"/>
+      <c r="O14" s="162"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="J15" s="155"/>
-      <c r="K15" s="156"/>
-      <c r="L15" s="157"/>
-      <c r="M15" s="159"/>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="L15" s="155"/>
+      <c r="M15" s="156"/>
+      <c r="N15" s="157"/>
+      <c r="O15" s="159"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="J16" s="155"/>
-      <c r="K16" s="156"/>
-      <c r="L16" s="157"/>
-      <c r="M16" s="163"/>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="L16" s="155"/>
+      <c r="M16" s="156"/>
+      <c r="N16" s="157"/>
+      <c r="O16" s="163"/>
     </row>
-    <row r="17" spans="10:13" x14ac:dyDescent="0.2">
-      <c r="J17" s="155"/>
-      <c r="K17" s="156"/>
-      <c r="L17" s="157"/>
-      <c r="M17" s="159"/>
+    <row r="17" spans="12:15" x14ac:dyDescent="0.2">
+      <c r="L17" s="155"/>
+      <c r="M17" s="156"/>
+      <c r="N17" s="157"/>
+      <c r="O17" s="159"/>
     </row>
-    <row r="18" spans="10:13" x14ac:dyDescent="0.2">
-      <c r="J18" s="157"/>
-      <c r="K18" s="158"/>
+    <row r="18" spans="12:15" x14ac:dyDescent="0.2">
       <c r="L18" s="157"/>
-      <c r="M18" s="159"/>
+      <c r="M18" s="158"/>
+      <c r="N18" s="157"/>
+      <c r="O18" s="159"/>
     </row>
-    <row r="19" spans="10:13" x14ac:dyDescent="0.2">
-      <c r="J19" s="155"/>
-      <c r="K19" s="159"/>
+    <row r="19" spans="12:15" x14ac:dyDescent="0.2">
+      <c r="L19" s="155"/>
+      <c r="M19" s="159"/>
     </row>
-    <row r="20" spans="10:13" x14ac:dyDescent="0.2">
-      <c r="J20" s="155"/>
-      <c r="K20" s="156"/>
+    <row r="20" spans="12:15" x14ac:dyDescent="0.2">
+      <c r="L20" s="155"/>
+      <c r="M20" s="156"/>
     </row>
-    <row r="21" spans="10:13" x14ac:dyDescent="0.2">
-      <c r="J21" s="155"/>
-      <c r="K21" s="156"/>
+    <row r="21" spans="12:15" x14ac:dyDescent="0.2">
+      <c r="L21" s="155"/>
+      <c r="M21" s="156"/>
     </row>
-    <row r="22" spans="10:13" x14ac:dyDescent="0.2">
-      <c r="J22" s="155"/>
-      <c r="K22" s="156"/>
+    <row r="22" spans="12:15" x14ac:dyDescent="0.2">
+      <c r="L22" s="155"/>
+      <c r="M22" s="156"/>
     </row>
-    <row r="23" spans="10:13" x14ac:dyDescent="0.2">
-      <c r="J23" s="155"/>
-      <c r="K23" s="156"/>
+    <row r="23" spans="12:15" x14ac:dyDescent="0.2">
+      <c r="L23" s="155"/>
+      <c r="M23" s="156"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
     <mergeCell ref="I3:I4"/>
     <mergeCell ref="J3:J4"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="L3:L4"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
Mejoras en dni de clientes uif y excel de flash AGG
</commit_message>
<xml_diff>
--- a/resources/templates/caja/flash/plantilla-flash-agg.xlsx
+++ b/resources/templates/caja/flash/plantilla-flash-agg.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="138">
   <si>
     <t>Consolidated Income</t>
   </si>
@@ -453,6 +453,9 @@
   </si>
   <si>
     <t>Ruletas</t>
+  </si>
+  <si>
+    <t>Total EP</t>
   </si>
 </sst>
 </file>
@@ -1517,7 +1520,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="45" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="338">
+  <cellXfs count="339">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -2172,6 +2175,7 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="171" fontId="12" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="47">
     <cellStyle name="20% - Accent1" xfId="22" builtinId="30" customBuiltin="1"/>
@@ -52407,24 +52411,30 @@
         <v>136</v>
       </c>
       <c r="D2" s="161" t="s">
+        <v>137</v>
+      </c>
+      <c r="E2" s="161" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="161"/>
       <c r="F2" s="161"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="155" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="156">
+      <c r="B3" s="338">
         <f>SUM(B4:B6)</f>
         <v>0</v>
       </c>
-      <c r="C3" s="156">
+      <c r="C3" s="338">
         <f>SUM(C4:C6)</f>
         <v>0</v>
       </c>
-      <c r="D3" s="156">
+      <c r="D3" s="338">
+        <f>SUM(D4:D6)</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="156">
         <f>HLOOKUP(J3,Resumen!BE5:BH39,+'Biyemas S.A.'!D1+2,0)</f>
         <v>0</v>
       </c>
@@ -52446,15 +52456,19 @@
       <c r="A4" s="155" t="s">
         <v>89</v>
       </c>
-      <c r="B4" s="156">
+      <c r="B4" s="338">
         <f>INDEX('Biyemas S.A.'!G7:G37,'Biyemas S.A.'!D1)</f>
         <v>0</v>
       </c>
-      <c r="C4" s="156">
+      <c r="C4" s="338">
         <f>INDEX('Biyemas S.A.'!O7:O37,'Biyemas S.A.'!D1)</f>
         <v>0</v>
       </c>
-      <c r="D4" s="156">
+      <c r="D4" s="338">
+        <f>SUM(B4,C4)</f>
+        <v>0</v>
+      </c>
+      <c r="E4" s="156">
         <f>HLOOKUP(J3,'Biyemas S.A.'!BE5:BH39,+'Biyemas S.A.'!D1+2,0)</f>
         <v>0</v>
       </c>
@@ -52468,15 +52482,19 @@
       <c r="A5" s="155" t="s">
         <v>90</v>
       </c>
-      <c r="B5" s="156">
+      <c r="B5" s="338">
         <f>INDEX('Kandiko S.A'!G7:G37,'Kandiko S.A'!D1)</f>
         <v>0</v>
       </c>
-      <c r="C5" s="156">
+      <c r="C5" s="338">
         <f>INDEX('Kandiko S.A'!O7:O37,'Kandiko S.A'!D1)</f>
         <v>0</v>
       </c>
-      <c r="D5" s="156">
+      <c r="D5" s="338">
+        <f>SUM(B5,C5)</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="156">
         <f>HLOOKUP(J3,'Kandiko S.A'!BA5:BF39,+'Biyemas S.A.'!D1+2,0)</f>
         <v>0</v>
       </c>
@@ -52486,15 +52504,19 @@
       <c r="A6" s="155" t="s">
         <v>91</v>
       </c>
-      <c r="B6" s="156">
+      <c r="B6" s="338">
         <f>INDEX('Rebisco S.A.'!G7:G37,'Rebisco S.A.'!D1)</f>
         <v>0</v>
       </c>
-      <c r="C6" s="156">
+      <c r="C6" s="338">
         <f>INDEX('Rebisco S.A.'!O7:O37,'Rebisco S.A.'!D1)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="156">
+      <c r="D6" s="338">
+        <f>SUM(B6,C6)</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="156">
         <f>HLOOKUP(J3,'Rebisco S.A.'!BA5:BF39,+'Biyemas S.A.'!D1+2,0)</f>
         <v>0</v>
       </c>
@@ -52519,12 +52541,15 @@
         <v>136</v>
       </c>
       <c r="D8" s="164" t="s">
+        <v>137</v>
+      </c>
+      <c r="E8" s="164" t="s">
         <v>87</v>
       </c>
-      <c r="E8" s="161" t="s">
+      <c r="F8" s="161" t="s">
         <v>118</v>
       </c>
-      <c r="F8" s="161" t="s">
+      <c r="G8" s="161" t="s">
         <v>119</v>
       </c>
       <c r="N8" s="157"/>
@@ -52534,23 +52559,27 @@
       <c r="A9" s="155" t="s">
         <v>88</v>
       </c>
-      <c r="B9" s="156">
+      <c r="B9" s="338">
         <f>SUM(B10:B12)</f>
         <v>0</v>
       </c>
-      <c r="C9" s="156">
+      <c r="C9" s="338">
         <f>SUM(C10:C12)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="156" t="e">
+      <c r="D9" s="338">
+        <f>SUM(D10:D12)</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="156" t="e">
         <f>+Resumen!BF39</f>
         <v>#N/A</v>
       </c>
-      <c r="E9" s="156" t="e">
+      <c r="F9" s="156" t="e">
         <f>+Resumen!AD48</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F9" s="156" t="e">
+      <c r="G9" s="156" t="e">
         <f>+Resumen!AD57</f>
         <v>#DIV/0!</v>
       </c>
@@ -52561,23 +52590,27 @@
       <c r="A10" s="155" t="s">
         <v>89</v>
       </c>
-      <c r="B10" s="156">
+      <c r="B10" s="338">
         <f>+'Biyemas S.A.'!G39</f>
         <v>0</v>
       </c>
-      <c r="C10" s="156">
+      <c r="C10" s="338">
         <f>+'Biyemas S.A.'!O39</f>
         <v>0</v>
       </c>
-      <c r="D10" s="156" t="e">
+      <c r="D10" s="338">
+        <f>SUM(B10,C10)</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="156" t="e">
         <f>+'Biyemas S.A.'!BF39</f>
         <v>#N/A</v>
       </c>
-      <c r="E10" s="156" t="e">
+      <c r="F10" s="156" t="e">
         <f>+'Biyemas S.A.'!AD48</f>
         <v>#N/A</v>
       </c>
-      <c r="F10" s="156" t="e">
+      <c r="G10" s="156" t="e">
         <f>+'Biyemas S.A.'!AD57</f>
         <v>#N/A</v>
       </c>
@@ -52588,23 +52621,27 @@
       <c r="A11" s="155" t="s">
         <v>90</v>
       </c>
-      <c r="B11" s="156">
+      <c r="B11" s="338">
         <f>+'Kandiko S.A'!G39</f>
         <v>0</v>
       </c>
-      <c r="C11" s="156">
+      <c r="C11" s="338">
         <f>+'Kandiko S.A'!O39</f>
         <v>0</v>
       </c>
-      <c r="D11" s="156" t="e">
+      <c r="D11" s="338">
+        <f>SUM(B11,C11)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="156" t="e">
         <f>+'Kandiko S.A'!BF39</f>
         <v>#N/A</v>
       </c>
-      <c r="E11" s="156" t="e">
+      <c r="F11" s="156" t="e">
         <f>+'Kandiko S.A'!AD48</f>
         <v>#N/A</v>
       </c>
-      <c r="F11" s="156" t="e">
+      <c r="G11" s="156" t="e">
         <f>+'Kandiko S.A'!AD57</f>
         <v>#N/A</v>
       </c>
@@ -52615,23 +52652,27 @@
       <c r="A12" s="155" t="s">
         <v>91</v>
       </c>
-      <c r="B12" s="156">
+      <c r="B12" s="338">
         <f>+'Rebisco S.A.'!G39</f>
         <v>0</v>
       </c>
-      <c r="C12" s="156">
+      <c r="C12" s="338">
         <f>+'Rebisco S.A.'!O39</f>
         <v>0</v>
       </c>
-      <c r="D12" s="156" t="e">
+      <c r="D12" s="338">
+        <f>SUM(B12,C12)</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="156" t="e">
         <f>+'Rebisco S.A.'!BF39</f>
         <v>#N/A</v>
       </c>
-      <c r="E12" s="156" t="e">
+      <c r="F12" s="156" t="e">
         <f>+'Rebisco S.A.'!AD48</f>
         <v>#N/A</v>
       </c>
-      <c r="F12" s="156" t="e">
+      <c r="G12" s="156" t="e">
         <f>+'Rebisco S.A.'!AD57</f>
         <v>#N/A</v>
       </c>

</xml_diff>

<commit_message>
LSD e imputación de conceptos de sueldos, contratos de venta, canon municipal, remesas e Interbanking.
Incluye asientos/solicitud de pago desde liquidación, tags de concepto de venta, unificación de clientes UIF, CBU en pagos, mejoras de cierre máquina/gastronomía y Flash AGG.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/resources/templates/caja/flash/plantilla-flash-agg.xlsx
+++ b/resources/templates/caja/flash/plantilla-flash-agg.xlsx
@@ -52381,26 +52381,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A2:O23"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="145" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="9.5546875" style="145" customWidth="1"/>
-    <col min="4" max="4" width="9.5546875" style="145" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" style="145" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.6640625" style="145" customWidth="1"/>
-    <col min="7" max="7" width="13.6640625" style="145" customWidth="1"/>
-    <col min="8" max="8" width="3.44140625" style="145" customWidth="1"/>
-    <col min="9" max="10" width="13.6640625" style="145" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="4.88671875" style="145" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="13.6640625" style="145" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="13.6640625" style="145" customWidth="1"/>
-    <col min="14" max="14" width="16.44140625" style="145" customWidth="1"/>
-    <col min="15" max="15" width="7" style="154" customWidth="1"/>
-    <col min="16" max="16384" width="11.44140625" style="145"/>
+    <col min="1" max="7" width="17.138671875" style="145" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="160" t="s">
         <v>92</v>
       </c>
@@ -52418,7 +52405,7 @@
       </c>
       <c r="F2" s="161"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="155" t="s">
         <v>88</v>
       </c>
@@ -52435,24 +52422,12 @@
         <v>0</v>
       </c>
       <c r="E3" s="156">
-        <f>HLOOKUP(J3,Resumen!BE5:BH39,+'Biyemas S.A.'!D1+2,0)</f>
+        <f>HLOOKUP("Electronic",Resumen!BE5:BH39,+'Biyemas S.A.'!D1+2,0)</f>
         <v>0</v>
       </c>
       <c r="F3" s="39"/>
-      <c r="I3" s="331" t="s">
-        <v>39</v>
-      </c>
-      <c r="J3" s="289" t="s">
-        <v>42</v>
-      </c>
-      <c r="K3" s="289" t="s">
-        <v>43</v>
-      </c>
-      <c r="L3" s="333" t="s">
-        <v>44</v>
-      </c>
     </row>
-    <row r="4" spans="1:15" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="155" t="s">
         <v>89</v>
       </c>
@@ -52469,16 +52444,12 @@
         <v>0</v>
       </c>
       <c r="E4" s="156">
-        <f>HLOOKUP(J3,'Biyemas S.A.'!BE5:BH39,+'Biyemas S.A.'!D1+2,0)</f>
+        <f>HLOOKUP("Electronic",'Biyemas S.A.'!BE5:BH39,+'Biyemas S.A.'!D1+2,0)</f>
         <v>0</v>
       </c>
       <c r="F4" s="39"/>
-      <c r="I4" s="332"/>
-      <c r="J4" s="290"/>
-      <c r="K4" s="290"/>
-      <c r="L4" s="334"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="155" t="s">
         <v>90</v>
       </c>
@@ -52495,12 +52466,12 @@
         <v>0</v>
       </c>
       <c r="E5" s="156">
-        <f>HLOOKUP(J3,'Kandiko S.A'!BA5:BF39,+'Biyemas S.A.'!D1+2,0)</f>
+        <f>HLOOKUP("Electronic",'Kandiko S.A'!BA5:BF39,+'Biyemas S.A.'!D1+2,0)</f>
         <v>0</v>
       </c>
       <c r="F5" s="39"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="155" t="s">
         <v>91</v>
       </c>
@@ -52517,12 +52488,12 @@
         <v>0</v>
       </c>
       <c r="E6" s="156">
-        <f>HLOOKUP(J3,'Rebisco S.A.'!BA5:BF39,+'Biyemas S.A.'!D1+2,0)</f>
+        <f>HLOOKUP("Electronic",'Rebisco S.A.'!BA5:BF39,+'Biyemas S.A.'!D1+2,0)</f>
         <v>0</v>
       </c>
       <c r="F6" s="39"/>
     </row>
-    <row r="7" spans="1:15" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="157"/>
       <c r="B7" s="158"/>
       <c r="C7" s="158"/>
@@ -52530,7 +52501,7 @@
       <c r="E7" s="158"/>
       <c r="F7" s="39"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="160" t="s">
         <v>93</v>
       </c>
@@ -52552,10 +52523,8 @@
       <c r="G8" s="161" t="s">
         <v>119</v>
       </c>
-      <c r="N8" s="157"/>
-      <c r="O8" s="162"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="155" t="s">
         <v>88</v>
       </c>
@@ -52583,10 +52552,8 @@
         <f>+Resumen!AD57</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="N9" s="157"/>
-      <c r="O9" s="163"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="155" t="s">
         <v>89</v>
       </c>
@@ -52614,10 +52581,8 @@
         <f>+'Biyemas S.A.'!AD57</f>
         <v>#N/A</v>
       </c>
-      <c r="N10" s="157"/>
-      <c r="O10" s="163"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="155" t="s">
         <v>90</v>
       </c>
@@ -52645,10 +52610,8 @@
         <f>+'Kandiko S.A'!AD57</f>
         <v>#N/A</v>
       </c>
-      <c r="N11" s="157"/>
-      <c r="O11" s="163"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="155" t="s">
         <v>91</v>
       </c>
@@ -52676,78 +52639,13 @@
         <f>+'Rebisco S.A.'!AD57</f>
         <v>#N/A</v>
       </c>
-      <c r="N12" s="157"/>
-      <c r="O12" s="163"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="39"/>
       <c r="D13" s="39"/>
       <c r="E13" s="39"/>
-      <c r="L13" s="160"/>
-      <c r="M13" s="161"/>
-      <c r="N13" s="157"/>
-      <c r="O13" s="159"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="L14" s="155"/>
-      <c r="M14" s="156"/>
-      <c r="N14" s="157"/>
-      <c r="O14" s="162"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="L15" s="155"/>
-      <c r="M15" s="156"/>
-      <c r="N15" s="157"/>
-      <c r="O15" s="159"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="L16" s="155"/>
-      <c r="M16" s="156"/>
-      <c r="N16" s="157"/>
-      <c r="O16" s="163"/>
-    </row>
-    <row r="17" spans="12:15" x14ac:dyDescent="0.2">
-      <c r="L17" s="155"/>
-      <c r="M17" s="156"/>
-      <c r="N17" s="157"/>
-      <c r="O17" s="159"/>
-    </row>
-    <row r="18" spans="12:15" x14ac:dyDescent="0.2">
-      <c r="L18" s="157"/>
-      <c r="M18" s="158"/>
-      <c r="N18" s="157"/>
-      <c r="O18" s="159"/>
-    </row>
-    <row r="19" spans="12:15" x14ac:dyDescent="0.2">
-      <c r="L19" s="155"/>
-      <c r="M19" s="159"/>
-    </row>
-    <row r="20" spans="12:15" x14ac:dyDescent="0.2">
-      <c r="L20" s="155"/>
-      <c r="M20" s="156"/>
-    </row>
-    <row r="21" spans="12:15" x14ac:dyDescent="0.2">
-      <c r="L21" s="155"/>
-      <c r="M21" s="156"/>
-    </row>
-    <row r="22" spans="12:15" x14ac:dyDescent="0.2">
-      <c r="L22" s="155"/>
-      <c r="M22" s="156"/>
-    </row>
-    <row r="23" spans="12:15" x14ac:dyDescent="0.2">
-      <c r="L23" s="155"/>
-      <c r="M23" s="156"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="J3:J4"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="L3:L4"/>
-  </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Mejoras en compras (legajo, pagos, sync Anita), gastronomía, mayor plano e IVA ventas.
Incluye asignación de factura a OC, firmante gastronomía, Interbanking, costos de insumos, cierre de período y migraciones asociadas.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/resources/templates/caja/flash/plantilla-flash-agg.xlsx
+++ b/resources/templates/caja/flash/plantilla-flash-agg.xlsx
@@ -41922,7 +41922,7 @@
         <v/>
       </c>
       <c r="BB7" s="181" t="str">
-        <f>IF(A7="","",IF($BA$7&gt;0,(C7-BA7)/BA7,))</f>
+        <f>IF(A7="","",IF(BA7&gt;0,(C7-BA7)/BA7,100%))</f>
         <v/>
       </c>
       <c r="BC7" s="176" t="str">
@@ -42186,7 +42186,7 @@
         <v/>
       </c>
       <c r="BB8" s="181" t="str">
-        <f t="shared" ref="BB8:BB38" si="21">IF(A8="","",IF($BA$7&gt;0,(C8-BA8)/BA8,))</f>
+        <f t="shared" ref="BB8:BB38" si="21">IF(A8="","",IF(BA8&gt;0,(C8-BA8)/BA8,100%))</f>
         <v/>
       </c>
       <c r="BC8" s="180" t="str">
@@ -50149,7 +50149,7 @@
         <v>0</v>
       </c>
       <c r="BB39" s="171">
-        <f>IF($AK39&gt;0,(C39-($BA39))/($BA$39),)</f>
+        <f>IF($AK39&gt;0,(C39-($BA39))/($BA$39),0)</f>
         <v>0</v>
       </c>
       <c r="BC39" s="175">
@@ -50855,7 +50855,7 @@
         <v>#N/A</v>
       </c>
       <c r="BB45" s="171" t="e">
-        <f>IF($AK45&gt;0,(C45-($BA45))/($BA$45),)</f>
+        <f>IF($AK45&gt;0,(C45-($BA45))/($BA$45),0)</f>
         <v>#N/A</v>
       </c>
       <c r="BC45" s="175" t="e">
@@ -51714,7 +51714,7 @@
         <v>#N/A</v>
       </c>
       <c r="BB54" s="171" t="e">
-        <f>IF($AK54&gt;0,(C54-($BA54))/($BA$54),)</f>
+        <f>IF($AK54&gt;0,(C54-($BA54))/($BA$54),0)</f>
         <v>#N/A</v>
       </c>
       <c r="BC54" s="175" t="e">

</xml_diff>